<commit_message>
update RG + canvas + k giới hạn đơn
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Auto PO Crea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5CE897-D959-40FC-88DC-763C451A1B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5148358-19BC-43C3-A080-14F4F5A59751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>SKU</t>
   </si>
@@ -33,44 +33,29 @@
     <t>Số lượng</t>
   </si>
   <si>
-    <t>12-6-200-110</t>
+    <t>50-26-150-72</t>
   </si>
   <si>
-    <t>12-3-200-110</t>
-  </si>
-  <si>
-    <t>13-6-200-110</t>
-  </si>
-  <si>
-    <t>11-6-200-110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5-6-200-110 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">5-3-200-110 </t>
-  </si>
-  <si>
-    <t>32-6-200-110</t>
-  </si>
-  <si>
-    <t>35-6-200-110</t>
-  </si>
-  <si>
-    <t>31-6-200-110</t>
+    <t>3-6-200-110</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF081B3A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,8 +78,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,7 +361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -389,12 +375,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -402,66 +388,11 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>